<commit_message>
Update Funds sent to Josh
</commit_message>
<xml_diff>
--- a/admin/resources/BeyondBordersReport-081126.xlsx
+++ b/admin/resources/BeyondBordersReport-081126.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2112d72604738b70/MasterFolder/Documents/JoshBeyondBorders/admin/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2112d72604738b70/MasterFolder/Documents/A_WebDev/JoshBeyondBorders/admin/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77C8E859-C1CE-4129-A095-325187A28052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{77C8E859-C1CE-4129-A095-325187A28052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6528A7CB-E4BF-40AE-8623-CA17CE55731F}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="12645" xr2:uid="{81427B8D-EAE8-41DF-821D-AA76386F6205}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" xr2:uid="{81427B8D-EAE8-41DF-821D-AA76386F6205}"/>
   </bookViews>
   <sheets>
     <sheet name="BeyondBordersReport" sheetId="1" r:id="rId1"/>
@@ -32,8 +32,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={F7691E2F-CE85-4FFF-96A5-3F22FE8992F1}</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{F7691E2F-CE85-4FFF-96A5-3F22FE8992F1}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This is the date that funds were transferred to Josh’s account. </t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="94">
   <si>
     <t>Time</t>
   </si>
@@ -312,13 +330,16 @@
   </si>
   <si>
     <t>Allen</t>
+  </si>
+  <si>
+    <t>Paid Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -453,8 +474,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -632,6 +659,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -795,10 +828,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -858,7 +892,9 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Brent Kern" id="{BA80F5D0-FD11-40B1-827C-E9B304798A36}" userId="2112d72604738b70" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1176,695 +1212,728 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A1" dT="2026-08-16T17:50:58.79" personId="{BA80F5D0-FD11-40B1-827C-E9B304798A36}" id="{F7691E2F-CE85-4FFF-96A5-3F22FE8992F1}">
+    <text xml:space="preserve">This is the date that funds were transferred to Josh’s account. </text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C2614E-98C5-436B-888A-5EBA73050BB5}">
-  <dimension ref="A1:AO8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C2614E-98C5-436B-888A-5EBA73050BB5}">
+  <dimension ref="A1:AP8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B2" s="1">
         <v>46239</v>
       </c>
-      <c r="B2" s="2">
+      <c r="C2" s="2">
         <v>0.68855324074074076</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>41</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>42</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>43</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>44</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>100</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>-2.48</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>97.52</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>45</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>46</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>47</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>48</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>49</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>51</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>0</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>0</v>
       </c>
-      <c r="AB2">
+      <c r="AC2">
         <v>1</v>
       </c>
-      <c r="AC2">
+      <c r="AD2">
         <v>1321926570971260</v>
       </c>
-      <c r="AD2">
+      <c r="AE2">
         <v>97.52</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>52</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>53</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AI2" t="s">
         <v>54</v>
       </c>
-      <c r="AI2">
+      <c r="AJ2">
         <v>75043</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
         <v>55</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AM2" t="s">
         <v>56</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AO2" t="s">
         <v>57</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AP2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B3" s="1">
         <v>46239</v>
       </c>
-      <c r="B3" s="2">
+      <c r="C3" s="2">
         <v>0.70478009259259256</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>40</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>59</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>42</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>43</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>44</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>100</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>-2.48</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>97.52</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>60</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>46</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>61</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>62</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>49</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>50</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>51</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>0</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>0</v>
       </c>
-      <c r="AB3">
+      <c r="AC3">
         <v>1</v>
       </c>
-      <c r="AD3">
+      <c r="AE3">
         <v>195.04</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AF3" t="s">
         <v>63</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AH3" t="s">
         <v>64</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AI3" t="s">
         <v>65</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AJ3" t="s">
         <v>66</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="AK3" t="s">
         <v>55</v>
       </c>
-      <c r="AK3">
+      <c r="AL3">
         <v>7814318771</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="AM3" t="s">
         <v>56</v>
       </c>
-      <c r="AN3" t="s">
+      <c r="AO3" t="s">
         <v>57</v>
       </c>
-      <c r="AO3" t="s">
+      <c r="AP3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B4" s="1">
         <v>46239</v>
       </c>
-      <c r="B4" s="2">
+      <c r="C4" s="2">
         <v>0.71960648148148143</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>40</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>67</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>42</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>43</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>44</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>200</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>-4.47</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>195.53</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>68</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>46</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>69</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>70</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>49</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>50</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>51</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>0</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>0</v>
       </c>
-      <c r="AB4">
+      <c r="AC4">
         <v>1</v>
       </c>
-      <c r="AD4">
+      <c r="AE4">
         <v>390.57</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AF4" t="s">
         <v>71</v>
       </c>
-      <c r="AG4" t="s">
+      <c r="AH4" t="s">
         <v>72</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AI4" t="s">
         <v>65</v>
       </c>
-      <c r="AI4">
+      <c r="AJ4">
         <v>1810</v>
       </c>
-      <c r="AJ4" t="s">
+      <c r="AK4" t="s">
         <v>55</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AM4" t="s">
         <v>56</v>
       </c>
-      <c r="AN4" t="s">
+      <c r="AO4" t="s">
         <v>57</v>
       </c>
-      <c r="AO4" t="s">
+      <c r="AP4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B5" s="1">
         <v>46239</v>
       </c>
-      <c r="B5" s="2">
+      <c r="C5" s="2">
         <v>0.76049768518518523</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>40</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>73</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>42</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>43</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>44</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>100</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>-3.48</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>96.52</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>74</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>46</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>76</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>49</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>50</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>51</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>0</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>0</v>
       </c>
-      <c r="AB5">
+      <c r="AC5">
         <v>1</v>
       </c>
-      <c r="AC5">
+      <c r="AD5">
         <v>163221723668187</v>
       </c>
-      <c r="AD5">
+      <c r="AE5">
         <v>291.56</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AF5" t="s">
         <v>77</v>
       </c>
-      <c r="AG5" t="s">
+      <c r="AH5" t="s">
         <v>78</v>
       </c>
-      <c r="AH5" t="s">
+      <c r="AI5" t="s">
         <v>65</v>
       </c>
-      <c r="AI5">
+      <c r="AJ5">
         <v>1453</v>
       </c>
-      <c r="AJ5" t="s">
+      <c r="AK5" t="s">
         <v>55</v>
       </c>
-      <c r="AL5" t="s">
+      <c r="AM5" t="s">
         <v>56</v>
       </c>
-      <c r="AN5" t="s">
+      <c r="AO5" t="s">
         <v>57</v>
       </c>
-      <c r="AO5" t="s">
+      <c r="AP5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B6" s="1">
         <v>46239</v>
       </c>
-      <c r="B6" s="2">
+      <c r="C6" s="2">
         <v>0.77787037037037032</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>40</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>79</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>42</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>43</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>100</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>-2.48</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>97.52</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>80</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>46</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>81</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>82</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>49</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>50</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>51</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>0</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>0</v>
       </c>
-      <c r="AB6">
+      <c r="AC6">
         <v>1</v>
       </c>
-      <c r="AD6">
+      <c r="AE6">
         <v>584.61</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="AF6" t="s">
         <v>83</v>
       </c>
-      <c r="AG6" t="s">
+      <c r="AH6" t="s">
         <v>84</v>
       </c>
-      <c r="AH6" t="s">
+      <c r="AI6" t="s">
         <v>65</v>
       </c>
-      <c r="AI6">
+      <c r="AJ6">
         <v>2176</v>
       </c>
-      <c r="AJ6" t="s">
+      <c r="AK6" t="s">
         <v>55</v>
       </c>
-      <c r="AL6" t="s">
+      <c r="AM6" t="s">
         <v>56</v>
       </c>
-      <c r="AN6" t="s">
+      <c r="AO6" t="s">
         <v>57</v>
       </c>
-      <c r="AO6" t="s">
+      <c r="AP6" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B7" s="1">
         <v>46241</v>
       </c>
-      <c r="B7" s="2">
+      <c r="C7" s="2">
         <v>0.88034722222222217</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>85</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>42</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>44</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>50</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>-1.49</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>48.51</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>86</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>46</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>87</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>88</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>49</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>50</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>51</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>0</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>0</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>89</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>90</v>
       </c>
-      <c r="AB7">
+      <c r="AC7">
         <v>1</v>
       </c>
-      <c r="AD7">
+      <c r="AE7">
         <v>535.6</v>
       </c>
-      <c r="AE7" t="s">
+      <c r="AF7" t="s">
         <v>91</v>
       </c>
-      <c r="AG7" t="s">
+      <c r="AH7" t="s">
         <v>92</v>
       </c>
-      <c r="AH7" t="s">
+      <c r="AI7" t="s">
         <v>54</v>
       </c>
-      <c r="AI7">
+      <c r="AJ7">
         <v>75013</v>
       </c>
-      <c r="AJ7" t="s">
+      <c r="AK7" t="s">
         <v>55</v>
       </c>
-      <c r="AL7" t="s">
+      <c r="AM7" t="s">
         <v>56</v>
       </c>
-      <c r="AN7" t="s">
+      <c r="AO7" t="s">
         <v>57</v>
       </c>
-      <c r="AO7" t="s">
+      <c r="AP7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="H8">
-        <f>SUM(H2:H7)</f>
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B8" s="1"/>
+      <c r="C8" s="2"/>
+      <c r="I8">
+        <f>SUM(I2:I7)</f>
         <v>650</v>
       </c>
-      <c r="J8">
-        <f>SUM(J2:J7)</f>
+      <c r="K8" s="3">
+        <f>SUM(K2:K7)</f>
         <v>633.12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change total to be the top row.
</commit_message>
<xml_diff>
--- a/admin/resources/BeyondBordersReport-081126.xlsx
+++ b/admin/resources/BeyondBordersReport-081126.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2112d72604738b70/MasterFolder/Documents/A_WebDev/JoshBeyondBorders/admin/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{77C8E859-C1CE-4129-A095-325187A28052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6528A7CB-E4BF-40AE-8623-CA17CE55731F}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{77C8E859-C1CE-4129-A095-325187A28052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B5E8EF7-1A35-4EC4-AEFC-2003E139AFD6}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" xr2:uid="{81427B8D-EAE8-41DF-821D-AA76386F6205}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="95">
   <si>
     <t>Time</t>
   </si>
@@ -333,13 +333,16 @@
   </si>
   <si>
     <t>Paid Date</t>
+  </si>
+  <si>
+    <t>Totals:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -473,12 +476,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1354,98 +1351,18 @@
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>46250</v>
-      </c>
-      <c r="B2" s="1">
-        <v>46239</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.68855324074074076</v>
-      </c>
-      <c r="D2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2" t="s">
-        <v>44</v>
-      </c>
-      <c r="I2">
-        <v>100</v>
-      </c>
-      <c r="J2">
-        <v>-2.48</v>
-      </c>
-      <c r="K2">
-        <v>97.52</v>
-      </c>
-      <c r="L2" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" t="s">
-        <v>46</v>
-      </c>
-      <c r="N2" t="s">
-        <v>47</v>
-      </c>
-      <c r="O2" t="s">
-        <v>48</v>
-      </c>
-      <c r="P2" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>50</v>
-      </c>
-      <c r="R2" t="s">
-        <v>51</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>1</v>
-      </c>
-      <c r="AD2">
-        <v>1321926570971260</v>
-      </c>
-      <c r="AE2">
-        <v>97.52</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>52</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>54</v>
-      </c>
-      <c r="AJ2">
-        <v>75043</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>55</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>57</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>58</v>
+      <c r="A2" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="I2" s="3">
+        <f>SUM(I3:I8)</f>
+        <v>650</v>
+      </c>
+      <c r="K2" s="3">
+        <f>SUM(K3:K1000)</f>
+        <v>633.12</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.25">
@@ -1456,13 +1373,13 @@
         <v>46239</v>
       </c>
       <c r="C3" s="2">
-        <v>0.70478009259259256</v>
+        <v>0.68855324074074076</v>
       </c>
       <c r="D3" t="s">
         <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="F3" t="s">
         <v>42</v>
@@ -1483,16 +1400,16 @@
         <v>97.52</v>
       </c>
       <c r="L3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="M3" t="s">
         <v>46</v>
       </c>
       <c r="N3" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="O3" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="P3" t="s">
         <v>49</v>
@@ -1512,26 +1429,26 @@
       <c r="AC3">
         <v>1</v>
       </c>
+      <c r="AD3">
+        <v>1321926570971260</v>
+      </c>
       <c r="AE3">
-        <v>195.04</v>
+        <v>97.52</v>
       </c>
       <c r="AF3" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="AH3" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="AI3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>66</v>
+        <v>54</v>
+      </c>
+      <c r="AJ3">
+        <v>75043</v>
       </c>
       <c r="AK3" t="s">
         <v>55</v>
-      </c>
-      <c r="AL3">
-        <v>7814318771</v>
       </c>
       <c r="AM3" t="s">
         <v>56</v>
@@ -1551,13 +1468,13 @@
         <v>46239</v>
       </c>
       <c r="C4" s="2">
-        <v>0.71960648148148143</v>
+        <v>0.70478009259259256</v>
       </c>
       <c r="D4" t="s">
         <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
         <v>42</v>
@@ -1569,25 +1486,25 @@
         <v>44</v>
       </c>
       <c r="I4">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J4">
-        <v>-4.47</v>
+        <v>-2.48</v>
       </c>
       <c r="K4">
-        <v>195.53</v>
+        <v>97.52</v>
       </c>
       <c r="L4" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="M4" t="s">
         <v>46</v>
       </c>
       <c r="N4" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="O4" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="P4" t="s">
         <v>49</v>
@@ -1608,22 +1525,25 @@
         <v>1</v>
       </c>
       <c r="AE4">
-        <v>390.57</v>
+        <v>195.04</v>
       </c>
       <c r="AF4" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="AH4" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="AI4" t="s">
         <v>65</v>
       </c>
-      <c r="AJ4">
-        <v>1810</v>
+      <c r="AJ4" t="s">
+        <v>66</v>
       </c>
       <c r="AK4" t="s">
         <v>55</v>
+      </c>
+      <c r="AL4">
+        <v>7814318771</v>
       </c>
       <c r="AM4" t="s">
         <v>56</v>
@@ -1643,13 +1563,13 @@
         <v>46239</v>
       </c>
       <c r="C5" s="2">
-        <v>0.76049768518518523</v>
+        <v>0.71960648148148143</v>
       </c>
       <c r="D5" t="s">
         <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
         <v>42</v>
@@ -1661,25 +1581,25 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J5">
-        <v>-3.48</v>
+        <v>-4.47</v>
       </c>
       <c r="K5">
-        <v>96.52</v>
+        <v>195.53</v>
       </c>
       <c r="L5" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="M5" t="s">
         <v>46</v>
       </c>
       <c r="N5" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="O5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="P5" t="s">
         <v>49</v>
@@ -1699,23 +1619,20 @@
       <c r="AC5">
         <v>1</v>
       </c>
-      <c r="AD5">
-        <v>163221723668187</v>
-      </c>
       <c r="AE5">
-        <v>291.56</v>
+        <v>390.57</v>
       </c>
       <c r="AF5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="AH5" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="AI5" t="s">
         <v>65</v>
       </c>
       <c r="AJ5">
-        <v>1453</v>
+        <v>1810</v>
       </c>
       <c r="AK5" t="s">
         <v>55</v>
@@ -1738,13 +1655,13 @@
         <v>46239</v>
       </c>
       <c r="C6" s="2">
-        <v>0.77787037037037032</v>
+        <v>0.76049768518518523</v>
       </c>
       <c r="D6" t="s">
         <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F6" t="s">
         <v>42</v>
@@ -1759,22 +1676,22 @@
         <v>100</v>
       </c>
       <c r="J6">
-        <v>-2.48</v>
+        <v>-3.48</v>
       </c>
       <c r="K6">
-        <v>97.52</v>
+        <v>96.52</v>
       </c>
       <c r="L6" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="M6" t="s">
         <v>46</v>
       </c>
       <c r="N6" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="O6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="P6" t="s">
         <v>49</v>
@@ -1794,20 +1711,23 @@
       <c r="AC6">
         <v>1</v>
       </c>
+      <c r="AD6">
+        <v>163221723668187</v>
+      </c>
       <c r="AE6">
-        <v>584.61</v>
+        <v>291.56</v>
       </c>
       <c r="AF6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AI6" t="s">
         <v>65</v>
       </c>
       <c r="AJ6">
-        <v>2176</v>
+        <v>1453</v>
       </c>
       <c r="AK6" t="s">
         <v>55</v>
@@ -1827,16 +1747,16 @@
         <v>46250</v>
       </c>
       <c r="B7" s="1">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="C7" s="2">
-        <v>0.88034722222222217</v>
+        <v>0.77787037037037032</v>
       </c>
       <c r="D7" t="s">
         <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
         <v>42</v>
@@ -1848,25 +1768,25 @@
         <v>44</v>
       </c>
       <c r="I7">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="J7">
-        <v>-1.49</v>
+        <v>-2.48</v>
       </c>
       <c r="K7">
-        <v>48.51</v>
+        <v>97.52</v>
       </c>
       <c r="L7" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="M7" t="s">
         <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="O7" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="P7" t="s">
         <v>49</v>
@@ -1883,29 +1803,23 @@
       <c r="U7">
         <v>0</v>
       </c>
-      <c r="V7" t="s">
-        <v>89</v>
-      </c>
-      <c r="W7" t="s">
-        <v>90</v>
-      </c>
       <c r="AC7">
         <v>1</v>
       </c>
       <c r="AE7">
-        <v>535.6</v>
+        <v>584.61</v>
       </c>
       <c r="AF7" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="AH7" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="AI7" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="AJ7">
-        <v>75013</v>
+        <v>2176</v>
       </c>
       <c r="AK7" t="s">
         <v>55</v>
@@ -1921,15 +1835,101 @@
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="B8" s="1"/>
-      <c r="C8" s="2"/>
+      <c r="A8" s="1">
+        <v>46250</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.88034722222222217</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" t="s">
+        <v>44</v>
+      </c>
       <c r="I8">
-        <f>SUM(I2:I7)</f>
-        <v>650</v>
-      </c>
-      <c r="K8" s="3">
-        <f>SUM(K2:K7)</f>
-        <v>633.12</v>
+        <v>50</v>
+      </c>
+      <c r="J8">
+        <v>-1.49</v>
+      </c>
+      <c r="K8">
+        <v>48.51</v>
+      </c>
+      <c r="L8" t="s">
+        <v>86</v>
+      </c>
+      <c r="M8" t="s">
+        <v>46</v>
+      </c>
+      <c r="N8" t="s">
+        <v>87</v>
+      </c>
+      <c r="O8" t="s">
+        <v>88</v>
+      </c>
+      <c r="P8" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>50</v>
+      </c>
+      <c r="R8" t="s">
+        <v>51</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8" t="s">
+        <v>89</v>
+      </c>
+      <c r="W8" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC8">
+        <v>1</v>
+      </c>
+      <c r="AE8">
+        <v>535.6</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ8">
+        <v>75013</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>